<commit_message>
[auto-snapshot] 2026-04-27 16:00 | onda-hompage | 73 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강화군_헬스장.xlsx
+++ b/naver-place-crawler/results_health/강화군_헬스장.xlsx
@@ -417,16 +417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -564,12 +564,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>에이스짐</t>
+          <t>익스트림패션</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>acegym2@naver.com</t>
+          <t>place_simulation@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -577,12 +577,12 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 강화대로404번길 7 3층</t>
+          <t>인천광역시 강화군 강화읍 동문안길20번길 6</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://instagram.com/ace__gym?igshid=ye2mgag95d7j</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -613,17 +613,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -632,17 +632,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1768451605</t>
+          <t>1135791607</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1768451605</t>
+          <t>https://m.place.naver.com/place/1135791607</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -654,29 +654,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>우리동네 헬스/PT</t>
+          <t>에이스짐</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>subgymasan@naver.com</t>
+          <t>acegym2@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>032-937-9870</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 불은면 강화동로 587 1층</t>
+          <t>인천광역시 강화군 강화읍 강화대로404번길 7 3층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://instagram.com/ace__gym?igshid=ye2mgag95d7j</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -686,7 +682,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -707,17 +703,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="R3" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -726,17 +722,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2084651240</t>
+          <t>1768451605</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2084651240</t>
+          <t>https://m.place.naver.com/place/1768451605</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -748,29 +744,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>에스오짐2호점</t>
+          <t>우리동네 헬스/PT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>topten0@naver.com</t>
+          <t>subgymasan@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>032-934-2124</t>
+          <t>032-937-9870</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 중앙로 27 3층 S.O GYM 2호점</t>
+          <t>인천광역시 강화군 불은면 강화동로 587 1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://instagram.com/sogym_official2</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -780,7 +776,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -801,17 +797,17 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>139</v>
+        <v>14</v>
       </c>
       <c r="Q4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>151</v>
+        <v>15</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -820,17 +816,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1935773088</t>
+          <t>2084651240</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1935773088</t>
+          <t>https://m.place.naver.com/place/2084651240</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -842,29 +838,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>몸짱휘트니스클럽</t>
+          <t>맥스휘트니스클럽. 맥스PT샵</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>byy333@naver.com</t>
+          <t>on180102@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1419-9688</t>
+          <t>0507-1327-2830</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 선원면 중앙로 154 2충</t>
+          <t>인천광역시 강화군 강화읍 동문안길 9-1 4층</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/byy333</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -874,12 +870,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -899,13 +895,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -914,51 +910,47 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>21494529</t>
+          <t>1506476586</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/21494529</t>
+          <t>https://m.place.naver.com/place/1506476586</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>위너핏</t>
+          <t>ACE GYM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>boos66@naver.com</t>
+          <t>wsh09@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0507-1476-1622</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>인천광역시 강화군 강화읍 남문로 14 3층</t>
+          <t>인천광역시 강화군 강화읍 강화대로404번길 7</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/boos66</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -968,12 +960,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -989,36 +981,690 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>1944033879</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1944033879</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>밸런스L.G.O휘트니스</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>topten0@naver.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 선원면 중앙로210번길 25</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>19399506</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/19399506</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>스카이헬스클럽</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>rokmc9160@naver.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0507-1468-7831</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 관청길23번길 8 관청길23번길8 스카이헬스클럽</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>17</v>
+      </c>
+      <c r="R8" t="n">
+        <v>23</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>11847161</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/11847161</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>에스오짐 1호점</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>topten0@naver.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0507-1381-0814</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 강화대로 199 2층</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>11</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1342561169</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1342561169</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>몸짱휘트니스클럽</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>byy333@naver.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0507-1419-9688</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 선원면 중앙로 154 2충</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/byy333</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>O</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" t="n">
+        <v>10</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>21494529</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/21494529</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>에스오짐2호점</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>topten0@naver.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>032-934-2124</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 중앙로 27 3층 S.O GYM 2호점</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://instagram.com/sogym_official2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>139</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>12</v>
+      </c>
+      <c r="R11" t="n">
+        <v>151</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>1935773088</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1935773088</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>맥스 PT&amp;GT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>topten0@naver.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0507-1407-5359</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 동문안길 9-1 4층</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1296569152</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1296569152</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>위너핏</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>boos66@naver.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0507-1476-1622</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>인천광역시 강화군 강화읍 남문로 14 3층</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/boos66</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
         <v>203</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q13" t="n">
         <v>293</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R13" t="n">
         <v>496</v>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
         <is>
           <t>1895477243</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/1895477243</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>

</xml_diff>